<commit_message>
Update: Latest changes from development session (data, UI improvements)
</commit_message>
<xml_diff>
--- a/data/activity_log.xlsx
+++ b/data/activity_log.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E82"/>
+  <dimension ref="A1:E113"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2606,6 +2606,831 @@
         </is>
       </c>
     </row>
+    <row r="83">
+      <c r="A83" t="inlineStr">
+        <is>
+          <t>2026-07-03 12:46:10</t>
+        </is>
+      </c>
+      <c r="B83" t="inlineStr">
+        <is>
+          <t>__solo__</t>
+        </is>
+      </c>
+      <c r="C83" t="inlineStr">
+        <is>
+          <t>participant</t>
+        </is>
+      </c>
+      <c r="D83" t="inlineStr">
+        <is>
+          <t>game_created</t>
+        </is>
+      </c>
+      <c r="E83" t="inlineStr">
+        <is>
+          <t>pin=114951 quiz=citi-trivia bots=True</t>
+        </is>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" t="inlineStr">
+        <is>
+          <t>2026-07-03 12:46:10</t>
+        </is>
+      </c>
+      <c r="B84" t="inlineStr">
+        <is>
+          <t>QuizNinja</t>
+        </is>
+      </c>
+      <c r="C84" t="inlineStr">
+        <is>
+          <t>host</t>
+        </is>
+      </c>
+      <c r="D84" t="inlineStr">
+        <is>
+          <t>game_started</t>
+        </is>
+      </c>
+      <c r="E84" t="inlineStr">
+        <is>
+          <t>pin=114951 players=7</t>
+        </is>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" t="inlineStr">
+        <is>
+          <t>2026-07-03 12:46:19</t>
+        </is>
+      </c>
+      <c r="B85" t="inlineStr">
+        <is>
+          <t>QuizNinja</t>
+        </is>
+      </c>
+      <c r="C85" t="inlineStr">
+        <is>
+          <t>participant</t>
+        </is>
+      </c>
+      <c r="D85" t="inlineStr">
+        <is>
+          <t>answer_submitted</t>
+        </is>
+      </c>
+      <c r="E85" t="inlineStr">
+        <is>
+          <t>q=1 correct=True points=1616</t>
+        </is>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" t="inlineStr">
+        <is>
+          <t>2026-07-03 12:46:25</t>
+        </is>
+      </c>
+      <c r="B86" t="inlineStr">
+        <is>
+          <t>QuizNinja</t>
+        </is>
+      </c>
+      <c r="C86" t="inlineStr">
+        <is>
+          <t>participant</t>
+        </is>
+      </c>
+      <c r="D86" t="inlineStr">
+        <is>
+          <t>answer_submitted</t>
+        </is>
+      </c>
+      <c r="E86" t="inlineStr">
+        <is>
+          <t>q=2 correct=False points=0</t>
+        </is>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" t="inlineStr">
+        <is>
+          <t>2026-07-03 12:46:27</t>
+        </is>
+      </c>
+      <c r="B87" t="inlineStr">
+        <is>
+          <t>QuizNinja</t>
+        </is>
+      </c>
+      <c r="C87" t="inlineStr">
+        <is>
+          <t>participant</t>
+        </is>
+      </c>
+      <c r="D87" t="inlineStr">
+        <is>
+          <t>answer_submitted</t>
+        </is>
+      </c>
+      <c r="E87" t="inlineStr">
+        <is>
+          <t>q=3 correct=True points=2007</t>
+        </is>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" t="inlineStr">
+        <is>
+          <t>2026-07-03 12:46:30</t>
+        </is>
+      </c>
+      <c r="B88" t="inlineStr">
+        <is>
+          <t>QuizNinja</t>
+        </is>
+      </c>
+      <c r="C88" t="inlineStr">
+        <is>
+          <t>participant</t>
+        </is>
+      </c>
+      <c r="D88" t="inlineStr">
+        <is>
+          <t>answer_submitted</t>
+        </is>
+      </c>
+      <c r="E88" t="inlineStr">
+        <is>
+          <t>q=4 correct=False points=0</t>
+        </is>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" t="inlineStr">
+        <is>
+          <t>2026-07-03 12:59:45</t>
+        </is>
+      </c>
+      <c r="B89" t="inlineStr">
+        <is>
+          <t>__solo__</t>
+        </is>
+      </c>
+      <c r="C89" t="inlineStr">
+        <is>
+          <t>participant</t>
+        </is>
+      </c>
+      <c r="D89" t="inlineStr">
+        <is>
+          <t>game_created</t>
+        </is>
+      </c>
+      <c r="E89" t="inlineStr">
+        <is>
+          <t>pin=756224 quiz=citi-trivia bots=True</t>
+        </is>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" t="inlineStr">
+        <is>
+          <t>2026-07-03 12:59:45</t>
+        </is>
+      </c>
+      <c r="B90" t="inlineStr">
+        <is>
+          <t>QuizNinja</t>
+        </is>
+      </c>
+      <c r="C90" t="inlineStr">
+        <is>
+          <t>host</t>
+        </is>
+      </c>
+      <c r="D90" t="inlineStr">
+        <is>
+          <t>game_started</t>
+        </is>
+      </c>
+      <c r="E90" t="inlineStr">
+        <is>
+          <t>pin=756224 players=7</t>
+        </is>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" t="inlineStr">
+        <is>
+          <t>2026-07-03 13:00:42</t>
+        </is>
+      </c>
+      <c r="B91" t="inlineStr">
+        <is>
+          <t>__solo__</t>
+        </is>
+      </c>
+      <c r="C91" t="inlineStr">
+        <is>
+          <t>host</t>
+        </is>
+      </c>
+      <c r="D91" t="inlineStr">
+        <is>
+          <t>game_ended</t>
+        </is>
+      </c>
+      <c r="E91" t="inlineStr">
+        <is>
+          <t>pin=756224</t>
+        </is>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" t="inlineStr">
+        <is>
+          <t>2026-07-03 13:01:07</t>
+        </is>
+      </c>
+      <c r="B92" t="inlineStr">
+        <is>
+          <t>__solo__</t>
+        </is>
+      </c>
+      <c r="C92" t="inlineStr">
+        <is>
+          <t>participant</t>
+        </is>
+      </c>
+      <c r="D92" t="inlineStr">
+        <is>
+          <t>game_created</t>
+        </is>
+      </c>
+      <c r="E92" t="inlineStr">
+        <is>
+          <t>pin=111397 quiz=citi-trivia bots=True</t>
+        </is>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" t="inlineStr">
+        <is>
+          <t>2026-07-03 13:01:07</t>
+        </is>
+      </c>
+      <c r="B93" t="inlineStr">
+        <is>
+          <t>QuizNinja</t>
+        </is>
+      </c>
+      <c r="C93" t="inlineStr">
+        <is>
+          <t>host</t>
+        </is>
+      </c>
+      <c r="D93" t="inlineStr">
+        <is>
+          <t>game_started</t>
+        </is>
+      </c>
+      <c r="E93" t="inlineStr">
+        <is>
+          <t>pin=111397 players=7</t>
+        </is>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" t="inlineStr">
+        <is>
+          <t>2026-07-03 13:01:18</t>
+        </is>
+      </c>
+      <c r="B94" t="inlineStr">
+        <is>
+          <t>__solo__</t>
+        </is>
+      </c>
+      <c r="C94" t="inlineStr">
+        <is>
+          <t>host</t>
+        </is>
+      </c>
+      <c r="D94" t="inlineStr">
+        <is>
+          <t>game_ended</t>
+        </is>
+      </c>
+      <c r="E94" t="inlineStr">
+        <is>
+          <t>pin=111397</t>
+        </is>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" t="inlineStr">
+        <is>
+          <t>2026-07-03 13:02:09</t>
+        </is>
+      </c>
+      <c r="B95" t="inlineStr">
+        <is>
+          <t>admin@citi.com</t>
+        </is>
+      </c>
+      <c r="C95" t="inlineStr">
+        <is>
+          <t>admin</t>
+        </is>
+      </c>
+      <c r="D95" t="inlineStr">
+        <is>
+          <t>login_ok</t>
+        </is>
+      </c>
+      <c r="E95" t="inlineStr"/>
+    </row>
+    <row r="96">
+      <c r="A96" t="inlineStr">
+        <is>
+          <t>2026-07-03 13:03:55</t>
+        </is>
+      </c>
+      <c r="B96" t="inlineStr">
+        <is>
+          <t>admin@citi.com</t>
+        </is>
+      </c>
+      <c r="C96" t="inlineStr">
+        <is>
+          <t>admin</t>
+        </is>
+      </c>
+      <c r="D96" t="inlineStr">
+        <is>
+          <t>login_ok</t>
+        </is>
+      </c>
+      <c r="E96" t="inlineStr"/>
+    </row>
+    <row r="97">
+      <c r="A97" t="inlineStr">
+        <is>
+          <t>2026-07-03 13:04:18</t>
+        </is>
+      </c>
+      <c r="B97" t="inlineStr">
+        <is>
+          <t>admin@citi.com</t>
+        </is>
+      </c>
+      <c r="C97" t="inlineStr">
+        <is>
+          <t>admin</t>
+        </is>
+      </c>
+      <c r="D97" t="inlineStr">
+        <is>
+          <t>game_created</t>
+        </is>
+      </c>
+      <c r="E97" t="inlineStr">
+        <is>
+          <t>pin=317872 quiz=bank-260703-105649 bots=True</t>
+        </is>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" t="inlineStr">
+        <is>
+          <t>2026-07-03 13:04:54</t>
+        </is>
+      </c>
+      <c r="B98" t="inlineStr">
+        <is>
+          <t>admin@citi.com</t>
+        </is>
+      </c>
+      <c r="C98" t="inlineStr">
+        <is>
+          <t>host</t>
+        </is>
+      </c>
+      <c r="D98" t="inlineStr">
+        <is>
+          <t>game_started</t>
+        </is>
+      </c>
+      <c r="E98" t="inlineStr">
+        <is>
+          <t>pin=317872 players=6</t>
+        </is>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" t="inlineStr">
+        <is>
+          <t>2026-07-03 13:05:21</t>
+        </is>
+      </c>
+      <c r="B99" t="inlineStr">
+        <is>
+          <t>admin@citi.com</t>
+        </is>
+      </c>
+      <c r="C99" t="inlineStr">
+        <is>
+          <t>host</t>
+        </is>
+      </c>
+      <c r="D99" t="inlineStr">
+        <is>
+          <t>game_ended</t>
+        </is>
+      </c>
+      <c r="E99" t="inlineStr">
+        <is>
+          <t>pin=317872</t>
+        </is>
+      </c>
+    </row>
+    <row r="100">
+      <c r="A100" t="inlineStr">
+        <is>
+          <t>2026-07-03 13:06:37</t>
+        </is>
+      </c>
+      <c r="B100" t="inlineStr">
+        <is>
+          <t xml:space="preserve">admin@citi.com </t>
+        </is>
+      </c>
+      <c r="C100" t="inlineStr">
+        <is>
+          <t>admin</t>
+        </is>
+      </c>
+      <c r="D100" t="inlineStr">
+        <is>
+          <t>login_ok</t>
+        </is>
+      </c>
+      <c r="E100" t="inlineStr"/>
+    </row>
+    <row r="101">
+      <c r="A101" t="inlineStr">
+        <is>
+          <t>2026-07-03 13:07:12</t>
+        </is>
+      </c>
+      <c r="B101" t="inlineStr">
+        <is>
+          <t>admin@citi.com</t>
+        </is>
+      </c>
+      <c r="C101" t="inlineStr">
+        <is>
+          <t>admin</t>
+        </is>
+      </c>
+      <c r="D101" t="inlineStr">
+        <is>
+          <t>game_created</t>
+        </is>
+      </c>
+      <c r="E101" t="inlineStr">
+        <is>
+          <t>pin=721252 quiz=bank-260703-105649 bots=True</t>
+        </is>
+      </c>
+    </row>
+    <row r="102">
+      <c r="A102" t="inlineStr">
+        <is>
+          <t>2026-07-03 13:07:24</t>
+        </is>
+      </c>
+      <c r="B102" t="inlineStr">
+        <is>
+          <t>RJ</t>
+        </is>
+      </c>
+      <c r="C102" t="inlineStr">
+        <is>
+          <t>participant</t>
+        </is>
+      </c>
+      <c r="D102" t="inlineStr">
+        <is>
+          <t>joined_game</t>
+        </is>
+      </c>
+      <c r="E102" t="inlineStr">
+        <is>
+          <t>pin=721252 team=-</t>
+        </is>
+      </c>
+    </row>
+    <row r="103">
+      <c r="A103" t="inlineStr">
+        <is>
+          <t>2026-07-03 13:07:38</t>
+        </is>
+      </c>
+      <c r="B103" t="inlineStr">
+        <is>
+          <t>admin@citi.com</t>
+        </is>
+      </c>
+      <c r="C103" t="inlineStr">
+        <is>
+          <t>host</t>
+        </is>
+      </c>
+      <c r="D103" t="inlineStr">
+        <is>
+          <t>game_started</t>
+        </is>
+      </c>
+      <c r="E103" t="inlineStr">
+        <is>
+          <t>pin=721252 players=7</t>
+        </is>
+      </c>
+    </row>
+    <row r="104">
+      <c r="A104" t="inlineStr">
+        <is>
+          <t>2026-07-03 13:07:54</t>
+        </is>
+      </c>
+      <c r="B104" t="inlineStr">
+        <is>
+          <t>RJ</t>
+        </is>
+      </c>
+      <c r="C104" t="inlineStr">
+        <is>
+          <t>participant</t>
+        </is>
+      </c>
+      <c r="D104" t="inlineStr">
+        <is>
+          <t>answer_submitted</t>
+        </is>
+      </c>
+      <c r="E104" t="inlineStr">
+        <is>
+          <t>q=1 correct=False points=0</t>
+        </is>
+      </c>
+    </row>
+    <row r="105">
+      <c r="A105" t="inlineStr">
+        <is>
+          <t>2026-07-03 13:08:16</t>
+        </is>
+      </c>
+      <c r="B105" t="inlineStr">
+        <is>
+          <t>RJ</t>
+        </is>
+      </c>
+      <c r="C105" t="inlineStr">
+        <is>
+          <t>participant</t>
+        </is>
+      </c>
+      <c r="D105" t="inlineStr">
+        <is>
+          <t>answer_submitted</t>
+        </is>
+      </c>
+      <c r="E105" t="inlineStr">
+        <is>
+          <t>q=2 correct=True points=1627</t>
+        </is>
+      </c>
+    </row>
+    <row r="106">
+      <c r="A106" t="inlineStr">
+        <is>
+          <t>2026-07-03 13:08:46</t>
+        </is>
+      </c>
+      <c r="B106" t="inlineStr">
+        <is>
+          <t>RJ</t>
+        </is>
+      </c>
+      <c r="C106" t="inlineStr">
+        <is>
+          <t>participant</t>
+        </is>
+      </c>
+      <c r="D106" t="inlineStr">
+        <is>
+          <t>answer_submitted</t>
+        </is>
+      </c>
+      <c r="E106" t="inlineStr">
+        <is>
+          <t>q=3 correct=True points=1601</t>
+        </is>
+      </c>
+    </row>
+    <row r="107">
+      <c r="A107" t="inlineStr">
+        <is>
+          <t>2026-07-03 13:09:42</t>
+        </is>
+      </c>
+      <c r="B107" t="inlineStr">
+        <is>
+          <t>RJ</t>
+        </is>
+      </c>
+      <c r="C107" t="inlineStr">
+        <is>
+          <t>participant</t>
+        </is>
+      </c>
+      <c r="D107" t="inlineStr">
+        <is>
+          <t>answer_submitted</t>
+        </is>
+      </c>
+      <c r="E107" t="inlineStr">
+        <is>
+          <t>q=5 correct=False points=0</t>
+        </is>
+      </c>
+    </row>
+    <row r="108">
+      <c r="A108" t="inlineStr">
+        <is>
+          <t>2026-07-03 13:10:16</t>
+        </is>
+      </c>
+      <c r="B108" t="inlineStr">
+        <is>
+          <t>RJ</t>
+        </is>
+      </c>
+      <c r="C108" t="inlineStr">
+        <is>
+          <t>participant</t>
+        </is>
+      </c>
+      <c r="D108" t="inlineStr">
+        <is>
+          <t>subjective_answer</t>
+        </is>
+      </c>
+      <c r="E108" t="inlineStr">
+        <is>
+          <t>q=6</t>
+        </is>
+      </c>
+    </row>
+    <row r="109">
+      <c r="A109" t="inlineStr">
+        <is>
+          <t>2026-07-03 13:10:22</t>
+        </is>
+      </c>
+      <c r="B109" t="inlineStr">
+        <is>
+          <t>RJ</t>
+        </is>
+      </c>
+      <c r="C109" t="inlineStr">
+        <is>
+          <t>participant</t>
+        </is>
+      </c>
+      <c r="D109" t="inlineStr">
+        <is>
+          <t>vote_cast</t>
+        </is>
+      </c>
+      <c r="E109" t="inlineStr">
+        <is>
+          <t>for=NightOwl_Sam q=6</t>
+        </is>
+      </c>
+    </row>
+    <row r="110">
+      <c r="A110" t="inlineStr">
+        <is>
+          <t>2026-07-03 13:10:56</t>
+        </is>
+      </c>
+      <c r="B110" t="inlineStr">
+        <is>
+          <t>admin@citi.com</t>
+        </is>
+      </c>
+      <c r="C110" t="inlineStr">
+        <is>
+          <t>host</t>
+        </is>
+      </c>
+      <c r="D110" t="inlineStr">
+        <is>
+          <t>force_reveal</t>
+        </is>
+      </c>
+      <c r="E110" t="inlineStr">
+        <is>
+          <t>q=8</t>
+        </is>
+      </c>
+    </row>
+    <row r="111">
+      <c r="A111" t="inlineStr">
+        <is>
+          <t>2026-07-03 13:11:01</t>
+        </is>
+      </c>
+      <c r="B111" t="inlineStr">
+        <is>
+          <t>admin@citi.com</t>
+        </is>
+      </c>
+      <c r="C111" t="inlineStr">
+        <is>
+          <t>host</t>
+        </is>
+      </c>
+      <c r="D111" t="inlineStr">
+        <is>
+          <t>force_reveal</t>
+        </is>
+      </c>
+      <c r="E111" t="inlineStr">
+        <is>
+          <t>q=9</t>
+        </is>
+      </c>
+    </row>
+    <row r="112">
+      <c r="A112" t="inlineStr">
+        <is>
+          <t>2026-07-03 13:11:04</t>
+        </is>
+      </c>
+      <c r="B112" t="inlineStr">
+        <is>
+          <t>admin@citi.com</t>
+        </is>
+      </c>
+      <c r="C112" t="inlineStr">
+        <is>
+          <t>host</t>
+        </is>
+      </c>
+      <c r="D112" t="inlineStr">
+        <is>
+          <t>force_reveal</t>
+        </is>
+      </c>
+      <c r="E112" t="inlineStr">
+        <is>
+          <t>q=10</t>
+        </is>
+      </c>
+    </row>
+    <row r="113">
+      <c r="A113" t="inlineStr">
+        <is>
+          <t>2026-07-03 13:11:20</t>
+        </is>
+      </c>
+      <c r="B113" t="inlineStr">
+        <is>
+          <t>admin@citi.com</t>
+        </is>
+      </c>
+      <c r="C113" t="inlineStr">
+        <is>
+          <t>host</t>
+        </is>
+      </c>
+      <c r="D113" t="inlineStr">
+        <is>
+          <t>game_ended</t>
+        </is>
+      </c>
+      <c r="E113" t="inlineStr">
+        <is>
+          <t>pin=721252</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>